<commit_message>
feat: competitor tracking (Phase 5)
- Optional "Competitors" sheet in the workbook: Competitor Of (IMECO SKU), Brand, Product Name,
  MRP and the three marketplace links. Keys come from the first link (C:amazon:<ASIN>), so
  there is no SKU to invent. The sheet is refused, by row, for an unknown IMECO SKU, a row with
  no link or a repeated link. IMECO's own catalogue parses exactly as before.
- Competitors are scraped like any listing. products.brand / competitor_of mark them; a
  database without those columns still gets IMECO's prices and skips the competitors.
- Dashboard: Prices board, header counts and the other tabs stay IMECO-only. New Competitors
  tab: each IMECO product with its rivals, price gap per marketplace, ratings, and how often
  IMECO is the cheapest.
- Example workbook gains a sample Competitors sheet. New views formatted with Prettier.
</commit_message>
<xml_diff>
--- a/Docs/pricing link.example.xlsx
+++ b/Docs/pricing link.example.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Competitors" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -556,4 +561,89 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor Of</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MRP</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon Link</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Flipkart Link</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Blinkit Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EXAMPLE1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Example Rival</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rival Product | 50 Pulls</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>279</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0EXAMPLE9</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: one sheet for products, competitors and keywords
The workbook's first sheet can now hold everything, each product followed by its rivals:

  SKU | Product Name | MRP | ... Links ... | Keywords | Competitor Of | Brand

- A row with "Competitor Of" is a competitor of that SKU (above or below it); it needs no SKU.
- A product's Keywords cell (comma, semicolon or new-line separated) feeds the daily search;
  the 19 defaults are used until any keyword is typed.
- The three columns are optional: today's sheet reads exactly as before (checked against the
  original parser). Separate "Competitors" / "Keywords" sheets are still accepted, read by the
  same rules.
- Example workbook and the dashboard's help text show the one-sheet layout.
</commit_message>
<xml_diff>
--- a/Docs/pricing link.example.xlsx
+++ b/Docs/pricing link.example.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Competitors" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -432,6 +431,9 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,6 +492,21 @@
           <t>Blinkit Link</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor Of</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -534,112 +551,54 @@
           <t>https://blinkit.com/prn/-/prid/100001</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>example product keyword, another keyword</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Example Rival Product | 50 Pulls</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0EXAMPLE9</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>EXAMPLE1</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Example Rival</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>EXAMPLE2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Example Product Two - No Blinkit Listing</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C4" t="n">
         <v>199</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>179</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B000000002</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Competitor Of</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Product Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>MRP</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Amazon Link</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Flipkart Link</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Blinkit Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>EXAMPLE1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Example Rival</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Rival Product | 50 Pulls</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>279</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0EXAMPLE9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: competitors as columns on each product's row
The product sheet keeps its rows exactly; competitors are extra columns on the right:
Competitor N Brand / Name / Amazon Link / Flipkart Link / Blinkit Link, for as many N as there
are column groups.
- A competitor is tracked once any of its links is filled in; blank ones are skipped.
- Keys are C:<IMECO SKU>:<marketplace>:<listing id>, so one rival listing can be compared with
  several IMECO products; the same rival twice under one product is tracked once.
- The current sheet still parses exactly as before. The "Competitor Of" row form is still read.
- Example workbook and the Competitors tab's help show the column layout.
- .gitignore covers every working copy of the pricing sheet, not just one file name.
</commit_message>
<xml_diff>
--- a/Docs/pricing link.example.xlsx
+++ b/Docs/pricing link.example.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -431,9 +431,22 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,12 +512,77 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Competitor Of</t>
+          <t>Competitor 1 Brand</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Competitor 1 Name</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 1 Amazon Link</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 1 Flipkart Link</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 1 Blinkit Link</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 2 Brand</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 2 Name</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 2 Amazon Link</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 2 Flipkart Link</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 2 Blinkit Link</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 3 Brand</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 3 Name</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 3 Amazon Link</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 3 Flipkart Link</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor 3 Blinkit Link</t>
         </is>
       </c>
     </row>
@@ -556,47 +634,40 @@
           <t>example product keyword, another keyword</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Example Rival</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Rival Product | 50 Pulls</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0EXAMPLE9</t>
+        </is>
+      </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EXAMPLE2</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Example Rival Product | 50 Pulls</t>
-        </is>
+          <t>Example Product Two - No Blinkit Listing</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>199</v>
+      </c>
+      <c r="D3" t="n">
+        <v>179</v>
       </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0EXAMPLE9</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>EXAMPLE1</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Example Rival</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>EXAMPLE2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Example Product Two - No Blinkit Listing</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>199</v>
-      </c>
-      <c r="D4" t="n">
-        <v>179</v>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B000000002</t>
         </is>

</xml_diff>